<commit_message>
refactor(fgui): 删除 GameHot 侧 UGUI 界面栈
</commit_message>
<xml_diff>
--- a/Design/Excel/GameHot/Datas/Game/UI.xlsx
+++ b/Design/Excel/GameHot/Datas/Game/UI.xlsx
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.872727272727269" defaultRowHeight="14"/>
   <cols>
     <col width="8.872727272727269" customWidth="1" style="3" min="1" max="1"/>
@@ -1385,21 +1385,21 @@
     </row>
     <row r="10">
       <c r="B10" s="3" t="n">
-        <v>1</v>
+        <v>103</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>DialogForm</t>
+          <t>FairyDemoForm</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>弹出框</t>
+          <t>FairyGUI演示</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Hot/DialogForm</t>
+          <t>FairyGUI/FairyDemoForm</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1408,29 +1408,39 @@
         </is>
       </c>
       <c r="G10" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="3" t="b">
         <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Package1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>MainView</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>MenuForm</t>
+          <t>FairyInventoryForm</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>主菜单</t>
+          <t>FairyGUI背包界面</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Hot/MenuForm</t>
+          <t>FairyGUI/FairyInventoryForm</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1442,62 +1452,82 @@
         <v>0</v>
       </c>
       <c r="H11" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Package1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>InventoryView</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="3" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>SettingForm</t>
+          <t>FairyItemDetailForm</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>设置</t>
+          <t>FairyGUI物品详情浮动窗口</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Hot/SettingForm</t>
+          <t>FairyGUI/FairyItemDetailForm</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Pop</t>
         </is>
       </c>
       <c r="G12" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Package1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>ItemDetailWindow</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>AboutForm</t>
+          <t>FairyInventoryOverlayForm</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>关于</t>
+          <t>FairyGUI背包遮罩界面</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Hot/AboutForm</t>
+          <t>FairyGUI/FairyInventoryOverlayForm</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Pop</t>
         </is>
       </c>
       <c r="G13" s="3" t="b">
@@ -1506,166 +1536,12 @@
       <c r="H13" s="3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="3" t="n">
-        <v>103</v>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>FairyDemoForm</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI演示</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI/FairyDemoForm</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="H14" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Package1</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>MainView</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="3" t="n">
-        <v>104</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>FairyInventoryForm</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI背包界面</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI/FairyInventoryForm</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="H15" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Package1</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>InventoryView</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="3" t="n">
-        <v>105</v>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>FairyItemDetailForm</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI物品详情浮动窗口</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI/FairyItemDetailForm</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Pop</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Package1</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>ItemDetailWindow</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="3" t="n">
-        <v>106</v>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>FairyInventoryOverlayForm</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI背包遮罩界面</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>FairyGUI/FairyInventoryOverlayForm</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Pop</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="H17" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Package1</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>InventoryOverlayView</t>
         </is>

</xml_diff>

<commit_message>
feat(hot): GameHot DialogForm 迁移到 FairyGUI(阶段E第一批)
设计端:
- Package1 新增 Dialog 组件(640x360:遮罩/标题/消息 + 确认/取消/中立
  三按钮,src 引用 DialogConfirmButton),经 FGUI agent-bridge 插件队列
  (create_component/create_button)驱动编辑器创建并 publish;新增
  .claude/scripts/fgui_queue.sh 队列辅助脚本。
- UI ID 保持 1(DialogForm/Default/multi=true/pause=true),Luban UI.xlsx
  恢复 DialogForm 行并导出;descriptor/bytes/绑定(UIDialog)全链生成。

运行时:
- DialogParams 契约与旧 UGUI 等价(Mode/Title/Message/三回调/PauseGame/
  UserData);FairyDialogForm Presenter 按模式控制按钮可见与文本,回调触发
  后经 FairyDialogFlow 关闭窗体;关闭时恢复暂停。
- 修复共享层时序契约:OnViewReady 阶段 context.Form 尚未回填(GF OnInit
  之后才有),Presenter 保存 context 引用、关闭时再取。
- FairyDialogSmokeTest:三模式/三回调/多实例独立关闭/PauseGame 暂停恢复/
  窗体数回基线;GameHot Editor asmdef 补 GameFramework 引用。

验证:gen 105-106 编译 0 error/0 warning;Dialog 冒烟通过;停 PlayMode 后
FairyGUI 路径 Error 日志 0(一条 UXTool 编辑器 LocalizationLanguage
IndexOutOfRange 为既存编辑器工具问题,与本批无关)。

后续批次:MenuForm/SettingForm/AboutForm 照此模式;旧 UGUI DialogForm
代码已于 87128db8 删除,本批无需再删。
</commit_message>
<xml_diff>
--- a/Design/Excel/GameHot/Datas/Game/UI.xlsx
+++ b/Design/Excel/GameHot/Datas/Game/UI.xlsx
@@ -1,16 +1,56 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr autoCompressPictures="1"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="17800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView windowHeight="17800" tabRatio="600"/>
   </bookViews>
   <sheets>
-    <sheet name="UI界面" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="UI界面" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="0" refMode="A1" iterate="0" fullPrecision="0" calcCompleted="0" calcOnSave="0" concurrentCalc="0" forceFullCalc="0"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">FairyRuntimeInspectorForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">运行时调试面板</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FairyGUI/FairyRuntimeInspectorForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RuntimeInspector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Package1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RuntimeInspectorView</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DialogForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">对话框</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FairyGUI/Dialog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dialog</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18,145 +58,145 @@
   <numFmts count="0"/>
   <fonts count="20">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color theme="1"/>
-      <sz val="11"/>
+      <name val="宋体"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -456,161 +496,161 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1022,203 +1062,203 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.872727272727269" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.87272727272727" defaultRowHeight="14"/>
   <cols>
-    <col width="8.872727272727269" customWidth="1" style="3" min="1" max="1"/>
-    <col width="19.3727272727273" customWidth="1" style="3" min="2" max="2"/>
-    <col width="20.7545454545455" customWidth="1" style="3" min="3" max="3"/>
-    <col width="22" customWidth="1" style="3" min="4" max="4"/>
-    <col width="52.1818181818182" customWidth="1" style="3" min="5" max="5"/>
-    <col width="14.6272727272727" customWidth="1" style="3" min="6" max="6"/>
-    <col width="23.1272727272727" customWidth="1" style="3" min="7" max="7"/>
-    <col width="23" customWidth="1" style="3" min="8" max="8"/>
-    <col width="8.872727272727269" customWidth="1" style="3" min="9" max="16384"/>
+    <col min="1" max="1" width="8.87272727272727" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.3727272727273" style="3" customWidth="1"/>
+    <col min="3" max="3" width="20.7545454545455" style="3" customWidth="1"/>
+    <col min="4" max="4" width="22" style="3" customWidth="1"/>
+    <col min="5" max="5" width="52.1818181818182" style="3" customWidth="1"/>
+    <col min="6" max="6" width="14.6272727272727" style="3" customWidth="1"/>
+    <col min="7" max="7" width="23.1272727272727" style="3" customWidth="1"/>
+    <col min="8" max="8" width="23" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.87272727272727" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>##var</t>
+          <t xml:space="preserve">##var</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t xml:space="preserve">Id</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>CSName</t>
+          <t xml:space="preserve">CSName</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Desc</t>
+          <t xml:space="preserve">Desc</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>AssetName</t>
+          <t xml:space="preserve">AssetName</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>UIGroupName</t>
+          <t xml:space="preserve">UIGroupName</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>AllowMultiInstance</t>
+          <t xml:space="preserve">AllowMultiInstance</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>PauseCoveredUIForm</t>
+          <t xml:space="preserve">PauseCoveredUIForm</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>PackageName</t>
+          <t xml:space="preserve">PackageName</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>ComponentName</t>
+          <t xml:space="preserve">ComponentName</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>##type</t>
+          <t xml:space="preserve">##type</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>int</t>
+          <t xml:space="preserve">int</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>string&amp;group=ge</t>
+          <t xml:space="preserve">string&amp;group=ge</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>string&amp;group=ge</t>
+          <t xml:space="preserve">string&amp;group=ge</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>string#path=normalAny;UI/*.json</t>
+          <t xml:space="preserve">string#path=normalAny;UI/*.json</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>##</t>
+          <t xml:space="preserve">##</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>界面编号</t>
+          <t xml:space="preserve">界面编号</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>代码名（程序填）</t>
+          <t xml:space="preserve">代码名（程序填）</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t xml:space="preserve">备注</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>资源名称</t>
+          <t xml:space="preserve">资源名称</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>界面组名称</t>
+          <t xml:space="preserve">界面组名称</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>是否允许多个界面实例</t>
+          <t xml:space="preserve">是否允许多个界面实例</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>是否暂停被其覆盖的界面</t>
+          <t xml:space="preserve">是否暂停被其覆盖的界面</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>包名</t>
+          <t xml:space="preserve">包名</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>组件名</t>
+          <t xml:space="preserve">组件名</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="3">
         <v>103</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>FairyDemoForm</t>
+          <t xml:space="preserve">FairyDemoForm</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI演示</t>
+          <t xml:space="preserve">FairyGUI演示</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyDemoForm</t>
+          <t xml:space="preserve">FairyGUI/FairyDemoForm</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t xml:space="preserve">Default</t>
         </is>
       </c>
       <c r="G4" s="3" t="b">
@@ -1229,37 +1269,37 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>MainView</t>
+          <t xml:space="preserve">MainView</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="3">
         <v>104</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>FairyInventoryForm</t>
+          <t xml:space="preserve">FairyInventoryForm</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI背包界面</t>
+          <t xml:space="preserve">FairyGUI背包界面</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyInventoryForm</t>
+          <t xml:space="preserve">FairyGUI/FairyInventoryForm</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t xml:space="preserve">Default</t>
         </is>
       </c>
       <c r="G5" s="3" t="b">
@@ -1270,37 +1310,37 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>InventoryView</t>
+          <t xml:space="preserve">InventoryView</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="3">
         <v>105</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>FairyItemDetailForm</t>
+          <t xml:space="preserve">FairyItemDetailForm</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI物品详情浮动窗口</t>
+          <t xml:space="preserve">FairyGUI物品详情浮动窗口</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyItemDetailForm</t>
+          <t xml:space="preserve">FairyGUI/FairyItemDetailForm</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Pop</t>
+          <t xml:space="preserve">Pop</t>
         </is>
       </c>
       <c r="G6" s="3" t="b">
@@ -1311,37 +1351,37 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>ItemDetailWindow</t>
+          <t xml:space="preserve">ItemDetailWindow</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="3">
         <v>106</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>FairyInventoryOverlayForm</t>
+          <t xml:space="preserve">FairyInventoryOverlayForm</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI背包遮罩界面</t>
+          <t xml:space="preserve">FairyGUI背包遮罩界面</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyInventoryOverlayForm</t>
+          <t xml:space="preserve">FairyGUI/FairyInventoryOverlayForm</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Pop</t>
+          <t xml:space="preserve">Pop</t>
         </is>
       </c>
       <c r="G7" s="3" t="b">
@@ -1352,37 +1392,37 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>InventoryOverlayView</t>
+          <t xml:space="preserve">InventoryOverlayView</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" t="n">
+      <c r="B8">
         <v>107</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FairyRuntimeInspectorForm</t>
+          <t xml:space="preserve">FairyRuntimeInspectorForm</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>运行时调试面板</t>
+          <t xml:space="preserve">运行时调试面板</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyRuntimeInspectorForm</t>
+          <t xml:space="preserve">FairyGUI/FairyRuntimeInspectorForm</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>RuntimeInspector</t>
+          <t xml:space="preserve">RuntimeInspector</t>
         </is>
       </c>
       <c r="G8" t="b">
@@ -1393,17 +1433,47 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>RuntimeInspectorView</t>
-        </is>
+          <t xml:space="preserve">RuntimeInspectorView</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>5</v>
+      </c>
+      <c r="J9" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
+  <sheetCalcPr fullCalcOnLoad="1"/>
   <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>